<commit_message>
tidy the design notebook: pacman, is.fullrank, plain spacing, and an overview sheet
</commit_message>
<xml_diff>
--- a/02_Differential_Expression/01_Design/c_data/01_design.xlsx
+++ b/02_Differential_Expression/01_Design/c_data/01_design.xlsx
@@ -7,7 +7,8 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="correlation_strata" sheetId="1" r:id="rId1"/>
+    <sheet name="overview" sheetId="1" r:id="rId1"/>
+    <sheet name="correlation_strata" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -351,6 +352,56 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>sheet</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>rows</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>columns</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>correlation_strata</t>
+        </is>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Consensus within-leg correlation with participant as a fixed term</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>

</xml_diff>